<commit_message>
Updated team contribution for sprint 2
</commit_message>
<xml_diff>
--- a/Sprint Planning/Product Backlog - SOEN 341.xlsx
+++ b/Sprint Planning/Product Backlog - SOEN 341.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagne\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF9703DF-2742-4BB7-AF0A-36E945CCA3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{455DBB0B-D2BC-4996-B66D-4A1450130EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{9FF516DD-DD1A-4540-862E-5B2452513E79}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="1" activeTab="2" xr2:uid="{9FF516DD-DD1A-4540-862E-5B2452513E79}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="69">
   <si>
     <t>The Cool Team</t>
   </si>
@@ -265,6 +265,11 @@
 Link the allergies/preferences to the user</t>
   </si>
   <si>
+    <t>Setup the recipe display page
+Improved UI for the display page
+Helped with "Add recipe"</t>
+  </si>
+  <si>
     <t>Created the GitHub, and helped fill out the product backlog.
 Setup the login and registration page.
 Setup the main menu and the profile page.
@@ -277,6 +282,28 @@
   <si>
     <t>found and setup the database and website host
 setup and debugged connectivity between website and database</t>
+  </si>
+  <si>
+    <t>Created acceptance tests for sprint 1 user stories
+Setup continuous integration pipeline</t>
+  </si>
+  <si>
+    <t>Added the recipe tables in the database
+Setup the add recipe function
+Helped with the recipe display
+Helped with the edit recipes
+Helped with the delete recipes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup the edit recipe function, and the remove recipe function. </t>
+  </si>
+  <si>
+    <t>Redesigned Recipes page layout
+Standardized styling across Add Recipe, Edit Recipe, and Recipes pages.
+Fixed Edit/Delete button alignment and styling</t>
+  </si>
+  <si>
+    <t>Setup the recipe filtering, sorting and searching</t>
   </si>
 </sst>
 </file>
@@ -1251,7 +1278,6 @@
     <mergeCell ref="F11:I11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1560,7 +1586,7 @@
         <v>46126</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="46">
         <v>11</v>
       </c>
@@ -1691,7 +1717,7 @@
     <col min="1" max="1" width="38.1796875" customWidth="1"/>
     <col min="2" max="2" width="31.54296875" customWidth="1"/>
     <col min="3" max="3" width="53.54296875" customWidth="1"/>
-    <col min="4" max="4" width="48.7265625" customWidth="1"/>
+    <col min="4" max="4" width="57.26953125" customWidth="1"/>
     <col min="5" max="5" width="47.7265625" customWidth="1"/>
     <col min="6" max="6" width="62.81640625" customWidth="1"/>
   </cols>
@@ -1724,12 +1750,14 @@
       <c r="C3" s="14">
         <v>6</v>
       </c>
-      <c r="D3" s="14"/>
+      <c r="D3" s="14">
+        <v>4</v>
+      </c>
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
       <c r="G3" s="11">
         <f>SUM(C3:F3)</f>
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="97.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -1740,7 +1768,9 @@
       <c r="C4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="15"/>
+      <c r="D4" s="4" t="s">
+        <v>67</v>
+      </c>
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
       <c r="G4" s="12"/>
@@ -1753,17 +1783,19 @@
         <v>56</v>
       </c>
       <c r="C5" s="14">
-        <v>8</v>
-      </c>
-      <c r="D5" s="14"/>
+        <v>6</v>
+      </c>
+      <c r="D5" s="14">
+        <v>4</v>
+      </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
       <c r="G5" s="11">
         <f>SUM(C5:F5)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="66.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="66.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="64"/>
       <c r="B6" s="7" t="s">
         <v>57</v>
@@ -1771,7 +1803,9 @@
       <c r="C6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
       <c r="G6" s="12"/>
@@ -1786,23 +1820,27 @@
       <c r="C7" s="14">
         <v>10</v>
       </c>
-      <c r="D7" s="14"/>
+      <c r="D7" s="14">
+        <v>10</v>
+      </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="11">
         <f>SUM(C7:F7)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="66.650000000000006" customHeight="1" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="76.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="66"/>
       <c r="B8" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="15"/>
+        <v>61</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="E8" s="15"/>
       <c r="F8" s="15"/>
       <c r="G8" s="12"/>
@@ -1817,12 +1855,14 @@
       <c r="C9" s="14">
         <v>2</v>
       </c>
-      <c r="D9" s="14"/>
+      <c r="D9" s="14">
+        <v>4</v>
+      </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="11">
         <f>SUM(C9:F9)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1831,9 +1871,11 @@
         <v>57</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="15"/>
+        <v>62</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>68</v>
+      </c>
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
       <c r="G10" s="12"/>
@@ -1848,12 +1890,14 @@
       <c r="C11" s="16">
         <v>5</v>
       </c>
-      <c r="D11" s="16"/>
+      <c r="D11" s="16">
+        <v>4</v>
+      </c>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="11">
         <f>SUM(C11:F11)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -1862,9 +1906,11 @@
         <v>57</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="15"/>
+        <v>63</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="13"/>
@@ -1877,12 +1923,14 @@
         <v>56</v>
       </c>
       <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
+      <c r="D13" s="16">
+        <v>4</v>
+      </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="11">
         <f>SUM(C13:F13)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -1891,7 +1939,9 @@
         <v>57</v>
       </c>
       <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
+      <c r="D14" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
       <c r="G14" s="13"/>

</xml_diff>